<commit_message>
:cat: añado la matriz de trazabilidad (punto 1) completa
</commit_message>
<xml_diff>
--- a/docs/Matriz de Trazabilidad preparcial.xlsx
+++ b/docs/Matriz de Trazabilidad preparcial.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daniel.rayo-r\IdeaProjects\DOSW_ParcialT2_DanielRayo\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC8E89F-CA87-48E6-B0E0-587107786DF7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D22A573-C147-4555-9367-1D51544889EC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{5DB214C1-7511-4C7C-96A1-3F1C917BAB0D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="76">
   <si>
     <t>ID</t>
   </si>
@@ -60,9 +60,6 @@
     <t>F03</t>
   </si>
   <si>
-    <t>Listar productos (filtro categoría/nombre)</t>
-  </si>
-  <si>
     <t>F04</t>
   </si>
   <si>
@@ -81,25 +78,7 @@
     <t>F02, F03</t>
   </si>
   <si>
-    <t>Ver resumen del carrito</t>
-  </si>
-  <si>
     <t>F07</t>
-  </si>
-  <si>
-    <t>F08</t>
-  </si>
-  <si>
-    <t>F06, F02</t>
-  </si>
-  <si>
-    <t>Procesar pago (aprobado/rechazado)</t>
-  </si>
-  <si>
-    <t>F09</t>
-  </si>
-  <si>
-    <t>(Admin) Crear/Editar/Desactivar producto</t>
   </si>
   <si>
     <t>Alta</t>
@@ -169,47 +148,6 @@
     <t>Solo consulta datos, no modifica nada en la BD. Puedes llamarlo 100 veces y el servidor siempre queda en el mismo estado.</t>
   </si>
   <si>
-    <t>name - String
-category - String</t>
-  </si>
-  <si>
-    <t>id - UUID
-name - String
-category - String
-description - String
-price - Double
-stock - Integer
-images - List&lt;String&gt;
-status - Boolean</t>
-  </si>
-  <si>
-    <t>Solo retorna productos con status = true (activos)
-Si category no coincide con ninguna categoría válida → 400
-Si no hay productos → retorna lista vacía [], no un 404</t>
-  </si>
-  <si>
-    <t>Happy Path 200 OK
-Categoría inválida 400 Invalid category
-Sin token 401 Unauthorized</t>
-  </si>
-  <si>
-    <t>// REQUEST
-GET /api/v1/products?category=running&amp;name=nike
-// RESPONSE 200
-[
-  {
-    "id": "uuid-1234",
-    "name": "Nike Air Max",
-    "description": "Zapatilla running profesional",
-    "category": "running",
-    "price": 250000.00,
-    "stock": 15,
-    "images": ["url1.jpg", "url2.jpg"],
-    "status": true
-  }
-]]</t>
-  </si>
-  <si>
     <t>Happy Path 200 OK
 Producto no encontrado 404 Product not found
 Sin token 401 Unauthorized</t>
@@ -220,10 +158,6 @@
   </si>
   <si>
     <t>id - UUID - obligatorio</t>
-  </si>
-  <si>
-    <t>ProductId - UUID - obligatorio
-quantity - Integer - obligatorio</t>
   </si>
   <si>
     <t>cartId - UUID
@@ -247,31 +181,12 @@
 Sin token 401 Unauthorized</t>
   </si>
   <si>
-    <t>Solo consulta el estado actual del carrito sin modificar nada en la BD. Llamarlo N veces siempre devuelve el mismo resultado.</t>
-  </si>
-  <si>
-    <t>userId - UUID - obligatorio</t>
-  </si>
-  <si>
-    <t>El usuario debe estar autenticado
-Si el carrito está vacío retorna lista vacía [], no un 404</t>
-  </si>
-  <si>
-    <t>Happy Path 200 OK
-Carrito vacío 200 []
-Sin token 401 Unauthorized</t>
-  </si>
-  <si>
     <t>cartId - UUID - obligatorio paymentMethod - String - obligatorio</t>
   </si>
   <si>
     <t>orderId - UUID
 status - String
 total - Double transactionId - UUID</t>
-  </si>
-  <si>
-    <t>El carrito no puede estar vacío
-Todos los productos deben tener stock suficiente Usuario autenticado</t>
   </si>
   <si>
     <t>Happy Path 201 Order created successfull
@@ -287,122 +202,10 @@
     <t>orderId - UUID - obligatorio paymentStatus - String - obligatorio</t>
   </si>
   <si>
-    <t>La orden debe existir
-La orden debe estar en estado PENDING
-Si aprobado: actualizar stock de productos</t>
-  </si>
-  <si>
     <t>Pago aprobado 200 Payment approved successfully
 Pago rechazado 200 Payment rejected 
 Orden no existe 404 Order not found
 Sin token 401 Unauthorized</t>
-  </si>
-  <si>
-    <t>POST
-PUT
-PATCH</t>
-  </si>
-  <si>
-    <t>POST: NO PUT: SI
-PATCH: SI</t>
-  </si>
-  <si>
-    <t>POST crea un nuevo recurso cada vez. PUT reemplaza el recurso completo, llamarlo N veces produce el mismo resultado. PATCH solo cambia el estado activo/inactivo.</t>
-  </si>
-  <si>
-    <t>name - String - obligatorio description - String - obligatorio category - String - obligatorio
-price - Double - obligatorio
-stock - Integer - obligatorio
-images - List&lt;String&gt; - opcional</t>
-  </si>
-  <si>
-    <t>id - UUID
-name - String
-category - String
-price - Double
-stock - Integer
-status - Boolean</t>
-  </si>
-  <si>
-    <t>Happy Path 201 Product created 
-Datos inválidos 400 Invalid input 
-Sin permisos 403 Forbidden
-Sin token 401 Unauthorized</t>
-  </si>
-  <si>
-    <t>// REQUEST
-POST /api/v1/orders
-{
-  "cartId": "uuid-cart-01",
-  "paymentMethod": "CREDIT_CARD"
-}
-// RESPONSE 201
-{
-  "orderId": "uuid-order-01",
-  "status": "PENDING",
-  "total": 500000.00,
-  "transactionId": "uuid-tx-01"
-}</t>
-  </si>
-  <si>
-    <t>// REQUEST APROBADO
-PUT /api/v1/orders/uuid-order-01/payment
-{
-  "paymentStatus": "APPROVED"
-}
-// RESPONSE 200 - APROBADO
-{
-  "orderId": "uuid-order-01",
-  "status": "PAID",
-  "transactionId": "uuid-tx-01",
-  "message": "Payment approved successfully"
-}
-// RESPONSE 200 - RECHAZADO
-{
-  "orderId": "uuid-order-01",
-  "status": "REJECTED",
-  "message": "Payment rejected, please try again"
-}</t>
-  </si>
-  <si>
-    <t>Solo rol ADMIN puede acceder
-price debe ser mayor a 0
-stock no puede ser negativo
-category debe ser válida</t>
-  </si>
-  <si>
-    <t>// REQUEST CREAR
-POST /api/v1/products
-{
-  "name": "Nike Air Max",
-  "description": "Zapatilla running profesional",
-  "category": "running",
-  "price": 250000.00,
-  "stock": 15,
-  "images": ["url1.jpg", "url2.jpg"]
-}
-// RESPONSE 201
-{
-  "id": "uuid-1234",
-  "name": "Nike Air Max",
-  "description": "Zapatilla running profesional",
-  "category": "running",
-  "price": 250000.00,
-  "stock": 15,
-  "status": true
-}
-// REQUEST DESACTIVAR
-PATCH /api/v1/products/uuid-1234
-{
-  "status": false
-}
-// RESPONSE 200
-{
-  "id": "uuid-1234",
-  "name": "Nike Air Max",
-  "status": false,
-  "message": "Product deactivated successfully"
-}</t>
   </si>
   <si>
     <t>id - UUID
@@ -476,31 +279,6 @@
   "price": 2500.00,
   "stock": 15,
   "state": "disponible"
-}</t>
-  </si>
-  <si>
-    <t>cartId - UUID
-items - List
-subtotals - Double
-total - Double</t>
-  </si>
-  <si>
-    <t>// REQUEST
-GET /api/v1/cart
-Authorization: Bearer eyJhbGci...
-// RESPONSE 200
-{
-  "cartId": "uuid-cart-01",
-  "items": [
-    {
-      "productId": "uuid-1234",
-      "productName": "Cafe Latte",
-      "quantity": 2,
-      "unitPrice": 2500.00,
-      "subtotal": 5000.00
-    }
-  ],
-  "total": 5000.00
 }</t>
   </si>
   <si>
@@ -522,6 +300,102 @@
   </si>
   <si>
     <t>Iniciar proceso de pedido</t>
+  </si>
+  <si>
+    <t>Procesar pedido</t>
+  </si>
+  <si>
+    <t>// REQUEST APROBADO
+PUT /api/v1/orders/uuid-order-01/payment
+{
+  "paymentStatus": "APPROVED"
+}
+// RESPONSE 200 - APROBADO
+{
+  "orderId": "uuid-order-01",
+  "status": "CREADO",
+  "transactionId": "uuid-tx-01",
+  "message": "Payment approved successfully"
+}
+// RESPONSE 200 - RECHAZADO
+{
+  "orderId": "uuid-order-01",
+  "status": "CANCELADO",
+  "message": "Payment rejected, please try again"
+}</t>
+  </si>
+  <si>
+    <t>La orden debe existir
+La orden debe crearse en estado CREADO
+Si aprobado: actualizar stock de productos</t>
+  </si>
+  <si>
+    <t>productId - UUID - obligatorio
+quantity - Integer - obligatorio</t>
+  </si>
+  <si>
+    <t>orderId - UUID - obligatorio
+status - String</t>
+  </si>
+  <si>
+    <t>id - UUID
+status - String</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+// REQUEST DESACTIVAR
+PATCH /api/v1/orders/uuid-order-01
+{
+  "status": "EN_PREPARACION"
+}
+// RESPONSE 200
+{
+  "id": "uuid-order-01", "message": "Product setted succesfully as EN_PREPARACION"
+}</t>
+  </si>
+  <si>
+    <t>Solo rol ADMIN puede acceder</t>
+  </si>
+  <si>
+    <t>Datos inválidos 400 Invalid input 
+Sin permisos 403 Forbidden
+Sin token 401 Unauthorized</t>
+  </si>
+  <si>
+    <t>(Admin) Editar Pedido</t>
+  </si>
+  <si>
+    <t>PATCH</t>
+  </si>
+  <si>
+    <t>PATCH solo cambia el estado EN_PREPARACION, ENTREGADO</t>
+  </si>
+  <si>
+    <t>// REQUEST
+POST /api/v1/orders
+{
+  "cartId": "uuid-cart-01",
+  "paymentMethod": "CREDIT_CARD"
+}
+// RESPONSE 201
+{
+  "orderId": "uuid-order-01",
+  "status": "CREADO",
+  "total": 5000.00,
+  "transactionId": "uuid-tx-01"
+}</t>
+  </si>
+  <si>
+    <t>El carrito no puede estar vacío
+Todos los productos deben tener stock suficiente
+El Usuario debe estar autenticado
+El pedido se crea en estado CREADO</t>
+  </si>
+  <si>
+    <t>F01, F02</t>
+  </si>
+  <si>
+    <t>F03, F04, F07</t>
   </si>
 </sst>
 </file>
@@ -550,7 +424,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -565,18 +439,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -696,17 +564,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -734,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -770,23 +627,18 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1035,8 +887,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{FBFD8D28-09BB-43FB-AA25-BFD458980327}" name="Tabla3" displayName="Tabla3" ref="B3:N12" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5">
-  <autoFilter ref="B3:N12" xr:uid="{FBFD8D28-09BB-43FB-AA25-BFD458980327}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{FBFD8D28-09BB-43FB-AA25-BFD458980327}" name="Tabla3" displayName="Tabla3" ref="B3:N10" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5">
+  <autoFilter ref="B3:N10" xr:uid="{FBFD8D28-09BB-43FB-AA25-BFD458980327}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{D13A3455-E4D4-4874-9BE7-BDB0A8FE4B33}" name="ID" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{E317DCBF-B1A0-4325-B0BC-4243E9125B4C}" name="Funcionalidad" dataDxfId="3"/>
@@ -1353,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B33B1AC-27C5-4B9B-8094-E12FC0724D74}">
-  <dimension ref="A3:N12"/>
+  <dimension ref="A3:N10"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
@@ -1386,32 +1238,32 @@
         <v>4</v>
       </c>
       <c r="G3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="255" x14ac:dyDescent="0.25">
-      <c r="A4" s="19"/>
+      <c r="A4" s="16"/>
       <c r="B4" s="8" t="s">
         <v>5</v>
       </c>
@@ -1419,39 +1271,41 @@
         <v>6</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="4"/>
+        <v>18</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="F4" s="10" t="s">
         <v>7</v>
       </c>
       <c r="G4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="J4" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="L4" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="M4" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="N4" s="16" t="s">
-        <v>38</v>
+        <v>29</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="N4" s="15" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="210" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
+      <c r="A5" s="16"/>
       <c r="B5" s="9" t="s">
         <v>8</v>
       </c>
@@ -1459,328 +1313,247 @@
         <v>9</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="F5" s="11" t="s">
         <v>5</v>
       </c>
       <c r="G5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="M5" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="N5" s="15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+      <c r="A6" s="16"/>
+      <c r="B6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
         <v>35</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H6" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I6" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J6" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="L5" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="M5" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N5" s="16" t="s">
+      <c r="K6" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="L6" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="M6" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" s="15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+      <c r="A7" s="16"/>
+      <c r="B7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="K7" s="15" t="s">
         <v>41</v>
       </c>
+      <c r="L7" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="M7" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="N7" s="15" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="6" spans="1:14" ht="300" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
-      <c r="B6" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="11" t="s">
+    <row r="8" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+      <c r="A8" s="16"/>
+      <c r="B8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="L8" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="M8" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="N8" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16"/>
+      <c r="B9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" t="s">
-        <v>43</v>
-      </c>
-      <c r="I6" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="K6" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="L6" s="16" t="s">
+      <c r="F9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="L9" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="N9" s="15" t="s">
         <v>49</v>
-      </c>
-      <c r="M6" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="N6" s="16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="210" x14ac:dyDescent="0.25">
-      <c r="A7" s="19"/>
-      <c r="B7" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" t="s">
-        <v>42</v>
-      </c>
-      <c r="H7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I7" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="J7" t="s">
-        <v>52</v>
-      </c>
-      <c r="K7" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="L7" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="M7" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N7" s="16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="255" x14ac:dyDescent="0.25">
-      <c r="A8" s="19"/>
-      <c r="B8" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" t="s">
-        <v>36</v>
-      </c>
-      <c r="I8" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="J8" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="K8" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="L8" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M8" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="N8" s="16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="300" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
-      <c r="B9" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>42</v>
-      </c>
-      <c r="H9" t="s">
-        <v>43</v>
-      </c>
-      <c r="I9" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="J9" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="K9" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="L9" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="M9" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="N9" s="16" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="225" x14ac:dyDescent="0.25">
-      <c r="B10" s="9" t="s">
+      <c r="A10" s="16"/>
+      <c r="B10" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" t="s">
-        <v>35</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="E10" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="I10" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="J10" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="L10" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="N10" s="16" t="s">
+      <c r="I10" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="15" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" ht="375" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H11" t="s">
-        <v>36</v>
-      </c>
-      <c r="I11" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="J11" s="16" t="s">
+      <c r="K10" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="L10" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K11" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="L11" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="M11" s="16" t="s">
+      <c r="M10" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="N11" s="16" t="s">
+      <c r="N10" s="15" t="s">
         <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="G12" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="I12" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="J12" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="K12" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="L12" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="M12" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="N12" s="16" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>